<commit_message>
added pdf export and fixed calendar entries
</commit_message>
<xml_diff>
--- a/KZN Calendar 05 May 2026 -2026_2027.xlsx
+++ b/KZN Calendar 05 May 2026 -2026_2027.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KZN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KZNACalendar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2731B36C-4342-4F54-ABD8-299B22287CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FEAC804-C9F4-4BE6-A4B5-9271B6A9730D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar" sheetId="1" r:id="rId1"/>
@@ -1077,11 +1077,11 @@
     <xf numFmtId="0" fontId="25" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1549,7 +1549,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1"/>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="46" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="45"/>
@@ -1567,7 +1567,7 @@
       <c r="G2" s="45"/>
     </row>
     <row r="5" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="44" t="s">
         <v>185</v>
       </c>
       <c r="B5" s="45"/>
@@ -1842,7 +1842,7 @@
       <c r="G16" s="11"/>
     </row>
     <row r="18" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="46" t="s">
+      <c r="A18" s="44" t="s">
         <v>193</v>
       </c>
       <c r="B18" s="45"/>
@@ -2123,7 +2123,7 @@
       <c r="G29" s="11"/>
     </row>
     <row r="31" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="46" t="s">
+      <c r="A31" s="44" t="s">
         <v>194</v>
       </c>
       <c r="B31" s="45"/>
@@ -2422,7 +2422,7 @@
       <c r="G44" s="11"/>
     </row>
     <row r="46" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="46" t="s">
+      <c r="A46" s="44" t="s">
         <v>195</v>
       </c>
       <c r="B46" s="45"/>
@@ -2704,7 +2704,7 @@
       <c r="G57" s="11"/>
     </row>
     <row r="59" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="46" t="s">
+      <c r="A59" s="44" t="s">
         <v>196</v>
       </c>
       <c r="B59" s="45"/>
@@ -2987,7 +2987,7 @@
       <c r="G70" s="11"/>
     </row>
     <row r="72" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="46" t="s">
+      <c r="A72" s="44" t="s">
         <v>197</v>
       </c>
       <c r="B72" s="45"/>
@@ -3281,7 +3281,7 @@
       <c r="G85" s="11"/>
     </row>
     <row r="87" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="46" t="s">
+      <c r="A87" s="44" t="s">
         <v>198</v>
       </c>
       <c r="B87" s="45"/>
@@ -3561,7 +3561,7 @@
       <c r="G98" s="11"/>
     </row>
     <row r="100" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="46" t="s">
+      <c r="A100" s="44" t="s">
         <v>199</v>
       </c>
       <c r="B100" s="45"/>
@@ -3855,7 +3855,7 @@
       </c>
     </row>
     <row r="113" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="46" t="s">
+      <c r="A113" s="44" t="s">
         <v>200</v>
       </c>
       <c r="B113" s="45"/>
@@ -4104,7 +4104,7 @@
       </c>
     </row>
     <row r="124" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="46" t="s">
+      <c r="A124" s="44" t="s">
         <v>201</v>
       </c>
       <c r="B124" s="45"/>
@@ -4385,7 +4385,7 @@
       <c r="G135" s="11"/>
     </row>
     <row r="137" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="46" t="s">
+      <c r="A137" s="44" t="s">
         <v>202</v>
       </c>
       <c r="B137" s="45"/>
@@ -4660,7 +4660,7 @@
       <c r="G148" s="11"/>
     </row>
     <row r="150" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="46" t="s">
+      <c r="A150" s="44" t="s">
         <v>203</v>
       </c>
       <c r="B150" s="45"/>
@@ -4958,12 +4958,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A150:G150"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A124:G124"/>
-    <mergeCell ref="A87:G87"/>
-    <mergeCell ref="A137:G137"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="A100:G100"/>
     <mergeCell ref="A72:G72"/>
@@ -4972,6 +4966,12 @@
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="A150:G150"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A124:G124"/>
+    <mergeCell ref="A87:G87"/>
+    <mergeCell ref="A137:G137"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -4992,7 +4992,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="46" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="45"/>
@@ -5434,7 +5434,7 @@
         <v>30</v>
       </c>
       <c r="G29" s="40" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
rebuild calendar from updated Excel
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KZN Calendar 05 May 2026 -2026_2027.xlsx
+++ b/KZN Calendar 05 May 2026 -2026_2027.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\KZNACalendar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FEAC804-C9F4-4BE6-A4B5-9271B6A9730D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46B3DC9-0D1B-4273-AAA0-D9A1B28BCC95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendar" sheetId="1" r:id="rId1"/>
@@ -1077,11 +1077,11 @@
     <xf numFmtId="0" fontId="25" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1549,7 +1549,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1"/>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="44" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="45"/>
@@ -1567,7 +1567,7 @@
       <c r="G2" s="45"/>
     </row>
     <row r="5" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="46" t="s">
         <v>185</v>
       </c>
       <c r="B5" s="45"/>
@@ -1842,7 +1842,7 @@
       <c r="G16" s="11"/>
     </row>
     <row r="18" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="44" t="s">
+      <c r="A18" s="46" t="s">
         <v>193</v>
       </c>
       <c r="B18" s="45"/>
@@ -2123,7 +2123,7 @@
       <c r="G29" s="11"/>
     </row>
     <row r="31" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="44" t="s">
+      <c r="A31" s="46" t="s">
         <v>194</v>
       </c>
       <c r="B31" s="45"/>
@@ -2391,11 +2391,11 @@
       </c>
       <c r="F42" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=F41)*(EventsTable[End Date]&gt;=F41))), "")</f>
-        <v>• Beavers SC Championships</v>
+        <v/>
       </c>
       <c r="G42" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=G41)*(EventsTable[End Date]&gt;=G41))), "")</f>
-        <v>• Beavers SC Championships</v>
+        <v/>
       </c>
     </row>
     <row r="43" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -2422,7 +2422,7 @@
       <c r="G44" s="11"/>
     </row>
     <row r="46" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="44" t="s">
+      <c r="A46" s="46" t="s">
         <v>195</v>
       </c>
       <c r="B46" s="45"/>
@@ -2550,11 +2550,11 @@
       </c>
       <c r="F51" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=F50)*(EventsTable[End Date]&gt;=F50))), "")</f>
-        <v/>
+        <v>• Beavers SC Championships</v>
       </c>
       <c r="G51" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=G50)*(EventsTable[End Date]&gt;=G50))), "")</f>
-        <v/>
+        <v>• Beavers SC Championships</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -2704,7 +2704,7 @@
       <c r="G57" s="11"/>
     </row>
     <row r="59" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="44" t="s">
+      <c r="A59" s="46" t="s">
         <v>196</v>
       </c>
       <c r="B59" s="45"/>
@@ -2987,7 +2987,7 @@
       <c r="G70" s="11"/>
     </row>
     <row r="72" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="44" t="s">
+      <c r="A72" s="46" t="s">
         <v>197</v>
       </c>
       <c r="B72" s="45"/>
@@ -3281,7 +3281,7 @@
       <c r="G85" s="11"/>
     </row>
     <row r="87" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="44" t="s">
+      <c r="A87" s="46" t="s">
         <v>198</v>
       </c>
       <c r="B87" s="45"/>
@@ -3400,19 +3400,21 @@
       </c>
       <c r="D92" s="5" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=D91)*(EventsTable[End Date]&gt;=D91))), "")</f>
-        <v/>
+        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
       </c>
       <c r="E92" s="5" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=E91)*(EventsTable[End Date]&gt;=E91))), "")</f>
-        <v/>
+        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
       </c>
       <c r="F92" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=F91)*(EventsTable[End Date]&gt;=F91))), "")</f>
-        <v>• Baynsfield Seeding Swim 2 / KZNA Open Water Champs</v>
+        <v>• Baynsfield Seeding Swim 2 / KZNA Open Water Champs
+• KZN Premier Championships (Level 2 &amp; Above)</v>
       </c>
       <c r="G92" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=G91)*(EventsTable[End Date]&gt;=G91))), "")</f>
-        <v>• Baynsfield Seeding Swim 2 / KZNA Open Water Champs</v>
+        <v>• Baynsfield Seeding Swim 2 / KZNA Open Water Champs
+• KZN Premier Championships (Level 2 &amp; Above)</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -3441,7 +3443,7 @@
     <row r="94" spans="1:7" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=A93)*(EventsTable[End Date]&gt;=A93))), "")</f>
-        <v/>
+        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
       </c>
       <c r="B94" s="5" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=B93)*(EventsTable[End Date]&gt;=B93))), "")</f>
@@ -3449,24 +3451,23 @@
       </c>
       <c r="C94" s="6" t="str">
         <f t="array" ref="C94">IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=C93)*(EventsTable[End Date]&gt;=C93))), "")</f>
-        <v>• KZN Premier Championships (Level 2 &amp; Above)
-• Day of Reconciliation</v>
+        <v>• Day of Reconciliation</v>
       </c>
       <c r="D94" s="5" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=D93)*(EventsTable[End Date]&gt;=D93))), "")</f>
-        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
+        <v/>
       </c>
       <c r="E94" s="5" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=E93)*(EventsTable[End Date]&gt;=E93))), "")</f>
-        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
+        <v/>
       </c>
       <c r="F94" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=F93)*(EventsTable[End Date]&gt;=F93))), "")</f>
-        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
+        <v/>
       </c>
       <c r="G94" s="6" t="str">
         <f>IFERROR(_xlfn.TEXTJOIN(CHAR(10), TRUE, "• " &amp; _xlfn._xlws.FILTER(EventsTable[Event Name], (EventsTable[Start Date]&lt;=G93)*(EventsTable[End Date]&gt;=G93))), "")</f>
-        <v>• KZN Premier Championships (Level 2 &amp; Above)</v>
+        <v/>
       </c>
     </row>
     <row r="95" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -3561,7 +3562,7 @@
       <c r="G98" s="11"/>
     </row>
     <row r="100" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="44" t="s">
+      <c r="A100" s="46" t="s">
         <v>199</v>
       </c>
       <c r="B100" s="45"/>
@@ -3855,7 +3856,7 @@
       </c>
     </row>
     <row r="113" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="44" t="s">
+      <c r="A113" s="46" t="s">
         <v>200</v>
       </c>
       <c r="B113" s="45"/>
@@ -4104,7 +4105,7 @@
       </c>
     </row>
     <row r="124" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A124" s="44" t="s">
+      <c r="A124" s="46" t="s">
         <v>201</v>
       </c>
       <c r="B124" s="45"/>
@@ -4385,7 +4386,7 @@
       <c r="G135" s="11"/>
     </row>
     <row r="137" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="44" t="s">
+      <c r="A137" s="46" t="s">
         <v>202</v>
       </c>
       <c r="B137" s="45"/>
@@ -4660,7 +4661,7 @@
       <c r="G148" s="11"/>
     </row>
     <row r="150" spans="1:7" ht="35.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A150" s="44" t="s">
+      <c r="A150" s="46" t="s">
         <v>203</v>
       </c>
       <c r="B150" s="45"/>
@@ -4958,6 +4959,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A150:G150"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A124:G124"/>
+    <mergeCell ref="A87:G87"/>
+    <mergeCell ref="A137:G137"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="A100:G100"/>
     <mergeCell ref="A72:G72"/>
@@ -4966,12 +4973,6 @@
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A150:G150"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A124:G124"/>
-    <mergeCell ref="A87:G87"/>
-    <mergeCell ref="A137:G137"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -4992,7 +4993,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="44" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="45"/>
@@ -5602,10 +5603,10 @@
         <v>60</v>
       </c>
       <c r="B38" s="42">
-        <v>46263</v>
+        <v>46277</v>
       </c>
       <c r="C38" s="42">
-        <v>46264</v>
+        <v>46278</v>
       </c>
       <c r="D38" s="40" t="s">
         <v>61</v>
@@ -6192,10 +6193,10 @@
         <v>116</v>
       </c>
       <c r="B66" s="42">
-        <v>46372</v>
+        <v>46366</v>
       </c>
       <c r="C66" s="42">
-        <v>46376</v>
+        <v>46370</v>
       </c>
       <c r="D66" s="40" t="s">
         <v>117</v>

</xml_diff>